<commit_message>
added some placeholders in the chest list spreadsheet
</commit_message>
<xml_diff>
--- a/assets/chest_item_list.xlsx
+++ b/assets/chest_item_list.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20361"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{811DB0AC-EBAE-4857-B93B-5D52564665DA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,10 +19,128 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t>Drop Rate</t>
+  </si>
+  <si>
+    <t>scythe</t>
+  </si>
+  <si>
+    <t>sword1</t>
+  </si>
+  <si>
+    <t>sword2</t>
+  </si>
+  <si>
+    <t>sword3</t>
+  </si>
+  <si>
+    <t>bow1</t>
+  </si>
+  <si>
+    <t>bow2</t>
+  </si>
+  <si>
+    <t>halberd</t>
+  </si>
+  <si>
+    <t>hammer1</t>
+  </si>
+  <si>
+    <t>hammer2</t>
+  </si>
+  <si>
+    <t>trident</t>
+  </si>
+  <si>
+    <t>magic staff1</t>
+  </si>
+  <si>
+    <t>magic staff2</t>
+  </si>
+  <si>
+    <t>dagger1</t>
+  </si>
+  <si>
+    <t>dagger2</t>
+  </si>
+  <si>
+    <t>dagger3</t>
+  </si>
+  <si>
+    <t>battle axe</t>
+  </si>
+  <si>
+    <t>spear</t>
+  </si>
+  <si>
+    <t>armor1</t>
+  </si>
+  <si>
+    <t>armor2</t>
+  </si>
+  <si>
+    <t>armor3</t>
+  </si>
+  <si>
+    <t>armor4</t>
+  </si>
+  <si>
+    <t>armor5</t>
+  </si>
+  <si>
+    <t>armor6</t>
+  </si>
+  <si>
+    <t>armor7</t>
+  </si>
+  <si>
+    <t>armor8</t>
+  </si>
+  <si>
+    <t>armor9</t>
+  </si>
+  <si>
+    <t>armor10</t>
+  </si>
+  <si>
+    <t>armor11</t>
+  </si>
+  <si>
+    <t>armor12</t>
+  </si>
+  <si>
+    <t>armor13</t>
+  </si>
+  <si>
+    <t>armor14</t>
+  </si>
+  <si>
+    <t>armor15</t>
+  </si>
+  <si>
+    <t>armor16</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -49,8 +168,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +450,291 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="12.140625" customWidth="1"/>
+    <col min="2" max="2" width="10.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>3.0625</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B15">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>20</v>
+      </c>
+      <c r="B20">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+      <c r="B21">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>